<commit_message>
out of model directory
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -224,7 +224,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AThree" displayName="AThree" ref="A1:J10" headerRowCount="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AThree" displayName="AThree" ref="A1:J12" headerRowCount="1" totalsRowShown="0">
   <autoFilter ref="A1:J4"/>
   <tableColumns count="10">
     <tableColumn id="1" name="SELECTED"/>
@@ -636,7 +636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -877,7 +877,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -902,24 +902,74 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
+        <v>0</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
         <v>1</v>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>1000181</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>1</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>g</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>D511</t>
         </is>

</xml_diff>

<commit_message>
10 labels per control no
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="5520" yWindow="3960" windowWidth="27140" windowHeight="21480" tabRatio="600" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1050" yWindow="1035" windowWidth="26310" windowHeight="11295" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="A03" sheetId="1" state="visible" r:id="rId1"/>
@@ -21,20 +21,27 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
-      <name val="Aptos Narrow"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="12"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Aptos Narrow"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <b val="1"/>
       <color theme="0"/>
       <sz val="12"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <charset val="129"/>
+      <family val="3"/>
+      <sz val="8"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -89,7 +96,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="4">
     <dxf>
@@ -224,8 +231,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AThree" displayName="AThree" ref="A1:J10" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:J8"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AThree" displayName="AThree" ref="A1:J88" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A1:J68"/>
   <tableColumns count="10">
     <tableColumn id="1" name="SELECTED"/>
     <tableColumn id="2" name="MaterialCode"/>
@@ -243,7 +250,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ATwo" displayName="ATwo" ref="A1:E4" headerRowCount="1" totalsRowShown="0" headerRowDxfId="3" tableBorderDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ATwo" displayName="ATwo" ref="A1:E4" headerRowCount="1" totalsRowShown="0" headerRowDxfId="1" tableBorderDxfId="0">
   <autoFilter ref="A1:E4"/>
   <tableColumns count="5">
     <tableColumn id="1" name="SELECTED"/>
@@ -257,8 +264,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Component" displayName="Component" ref="A14:H16" headerRowCount="1" totalsRowShown="0" headerRowDxfId="1" tableBorderDxfId="0">
-  <autoFilter ref="A14:H16"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Component" displayName="Component" ref="A11:H13" headerRowCount="1" totalsRowShown="0" headerRowDxfId="3" tableBorderDxfId="2">
+  <autoFilter ref="A11:H13"/>
   <tableColumns count="8">
     <tableColumn id="1" name="SELECTED"/>
     <tableColumn id="2" name="ReservationItemNo"/>
@@ -274,8 +281,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="PO" displayName="PO" ref="A1:L4" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:L4"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="PO" displayName="PO" ref="A1:L2" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A1:L2"/>
   <tableColumns count="12">
     <tableColumn id="1" name="SELECTED"/>
     <tableColumn id="2" name="ProductionOrderNo"/>
@@ -636,16 +643,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <dimension ref="A1:J88"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="11.5546875" defaultRowHeight="17.25"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="18.5" customWidth="1" min="2" max="2"/>
+    <col width="18.44140625" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="15.6640625" customWidth="1" min="4" max="4"/>
     <col width="20.33203125" customWidth="1" min="5" max="5"/>
     <col width="16.33203125" customWidth="1" min="7" max="8"/>
-    <col width="15.83203125" customWidth="1" min="9" max="9"/>
+    <col width="15.77734375" customWidth="1" min="9" max="9"/>
     <col width="12.33203125" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -877,7 +884,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -902,24 +909,2174 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
+        <v>0</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>0</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>0</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>0</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>0</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>0</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>0</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>0</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>0</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>0</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>0</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>0</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>0</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>0</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>0</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>0</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>0</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>0</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>0</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>0</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>0</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>0</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>0</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>0</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>0</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>0</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>0</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>0</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>0</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>0</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>0</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>0</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>0</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>0</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>0</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>0</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>0</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>0</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>0</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>0</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>2603296081</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>0</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>2603296081</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>0</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>2603296081</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>0</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>2603296081</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>0</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>2603296081</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>0</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>2603296081</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>0</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>2603296081</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>0</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>2603296081</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>0</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>2603296081</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>0</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>2603296081</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>0</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>2603291255</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>0</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>2603291255</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>0</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>2603291255</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>0</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>2603291255</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>0</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>2603291255</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>0</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>2603291255</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>0</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>2603291255</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>0</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>2603291255</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>0</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>2603291255</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>0</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>2603291255</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
         <v>1</v>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>1000181</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>2603296168</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>1</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>2603296168</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>1</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>2603296168</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>1</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>2603296168</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>1</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>2603296168</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>1</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>2603296168</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>1</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>2603296168</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>1</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>2603296168</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>1</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>2603296168</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>1</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>2603296168</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>1</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>1000121</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>2603298707</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>g</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>1</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>1000121</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>2603298707</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>1</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>1000121</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>2603298707</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>1</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>1000121</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>2603298707</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>1</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>1000121</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>2603298707</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>1</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>1000121</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>2603298707</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>1</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>1000121</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>2603298707</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>1</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>1000121</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>2603298707</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>1</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>1000121</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>2603298707</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>1</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>1000121</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>2603298707</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
         <is>
           <t>D511</t>
         </is>
@@ -927,6 +3084,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" paperSize="9" horizontalDpi="150" verticalDpi="150"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
@@ -940,11 +3098,11 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="11.5546875" defaultRowHeight="17.25"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="14.6640625" customWidth="1" min="2" max="2"/>
-    <col width="22.5" customWidth="1" min="3" max="3"/>
+    <col width="22.44140625" customWidth="1" min="3" max="3"/>
     <col width="13.6640625" customWidth="1" min="4" max="4"/>
     <col width="18.6640625" customWidth="1" min="5" max="5"/>
   </cols>
@@ -1035,15 +3193,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <dimension ref="A1:L13"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="11.5546875" defaultRowHeight="17.25"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="19.5" customWidth="1" min="2" max="3"/>
+    <col width="19.44140625" customWidth="1" min="2" max="3"/>
     <col width="18" customWidth="1" min="4" max="5"/>
     <col width="20.33203125" customWidth="1" min="6" max="6"/>
     <col width="19.33203125" customWidth="1" min="7" max="7"/>
-    <col width="18.83203125" customWidth="1" min="8" max="8"/>
+    <col width="18.77734375" customWidth="1" min="8" max="8"/>
     <col width="15.6640625" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="21.33203125" customWidth="1" min="11" max="11"/>
@@ -1130,101 +3288,101 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
         <is>
           <t>SELECTED</t>
         </is>
       </c>
-      <c r="B14" s="1" t="inlineStr">
+      <c r="B11" s="1" t="inlineStr">
         <is>
           <t>ReservationItemNo</t>
         </is>
       </c>
-      <c r="C14" s="1" t="inlineStr">
+      <c r="C11" s="1" t="inlineStr">
         <is>
           <t>ItemNo</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>ComponentCode</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>ComponentUOM</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="G11" s="4" t="inlineStr">
         <is>
           <t>StorageLocation</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H11" s="4" t="inlineStr">
         <is>
           <t>ValidDecimalPointNo</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
+    <row r="12">
+      <c r="A12" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B15" s="2" t="n">
+      <c r="B12" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" t="n">
         <v>1000181</v>
       </c>
-      <c r="C15" s="2" t="n"/>
-      <c r="D15" t="n">
-        <v>1000181</v>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>g</t>
-        </is>
-      </c>
-      <c r="F15" t="n">
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
         <v>100</v>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>D511</t>
-        </is>
-      </c>
-      <c r="H15" t="n">
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="n">
+    <row r="13">
+      <c r="A13" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B16" s="2" t="n">
-        <v>1000181</v>
-      </c>
-      <c r="C16" s="2" t="n"/>
-      <c r="D16" t="n">
-        <v>1000181</v>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>g</t>
-        </is>
-      </c>
-      <c r="F16" t="n">
+      <c r="B13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" t="n">
+        <v>1000121</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
         <v>200</v>
       </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>D511</t>
-        </is>
-      </c>
-      <c r="H16" t="n">
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>D511</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1244,16 +3402,16 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:L3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="11.5546875" defaultRowHeight="17.25"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="17.1640625" customWidth="1" min="2" max="2"/>
-    <col width="13.1640625" customWidth="1" min="7" max="7"/>
+    <col width="17.109375" customWidth="1" min="2" max="2"/>
+    <col width="13.109375" customWidth="1" min="7" max="7"/>
     <col width="17" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="17.33203125" customWidth="1" min="10" max="10"/>
     <col width="16.6640625" customWidth="1" min="11" max="11"/>
-    <col width="25.1640625" customWidth="1" min="12" max="12"/>
+    <col width="25.109375" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>